<commit_message>
Self-serve concept synthesis + head-to-head deliverables (Tier C, 62.6/100)
PM synthesis of the self-serve CMMC SaaS variant: Objectives 62.6/100, Tier C
(Pass / Reposition), hard-constraint #5 TRIGGERED (funded strong-tech incumbents
FutureFeed/Vanta/Drata/Secureframe), with a documented two-directional red-team
that confirmed competition at 3 on named, already-shipped evidence.

- Plain-English dossier + one-page scorecard (.md/.txt/.docx) for the self-serve
  concept, with full council appendix.
- Master comparison sheet (.csv/.xlsx) updated to both concepts head-to-head:
  Muster operated 76/B vs. Muster Self-Serve 62.6/C.
- Recommendation: reposition (not tweak) — keep the A-grade forcing function and
  the small-sub customer, abandon the contested self-serve-software lane; lead
  candidate is the multi-prime flow-down / questionnaire-response wedge.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XXPX8jb3AAt9NV25SZFk3X
</commit_message>
<xml_diff>
--- a/deliverables/2026-06-21/scoreboard.xlsx
+++ b/deliverables/2026-06-21/scoreboard.xlsx
@@ -425,22 +425,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:O3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="48" customWidth="1" min="2" max="2"/>
-    <col width="23" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="37" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="34" customWidth="1" min="10" max="10"/>
-    <col width="24" customWidth="1" min="11" max="11"/>
-    <col width="15" customWidth="1" min="12" max="12"/>
-    <col width="48" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="36" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="12" max="12"/>
+    <col width="23" customWidth="1" min="13" max="13"/>
+    <col width="20" customWidth="1" min="14" max="14"/>
+    <col width="48" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -451,60 +453,70 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Delivery model</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Forcing-function type</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Objectives Score /100</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>CFO</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>CMO</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>COO</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Legal</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>CTO</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Competitive</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Lowest sub-score</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Legal risk-gate</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Tier</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Hard-constraint #5</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>What it is</t>
         </is>
@@ -513,67 +525,154 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Muster</t>
+          <t>Muster (operated)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>Managed / artifact-only service</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>Regulatory mandate + contractual flow-down (Type 1+2)</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>76</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>8.4</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>7.5</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>7.6</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>8.1</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>8.2</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>6.6</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>3 (Competitive: reach-down risk)</t>
-        </is>
-      </c>
       <c r="K2" t="inlineStr">
         <is>
+          <t>3 (Competitive: reach-down)</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
           <t>SERIOUS-BUT-MANAGEABLE</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>B (Promising)</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>Managed, artifact-only NIST 800-171/SPRS &amp; CMMC readiness for small defense subcontractors — fixed price, never touches CUI</t>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Not triggered</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Operated, artifact-only NIST 800-171/SPRS &amp; CMMC readiness; fixed price; never touches CUI; founder-led close + RP/CCP sign-off</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Muster Self-Serve</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Self-serve software (no human gate)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Regulatory mandate + contractual flow-down (Type 1+2)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>62.6</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>8.3</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>6.9</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>8.0</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>8.2</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>7.4</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>4.4</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>2 (Competitive: reach-down SEVERE)</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>SERIOUS-BUT-MANAGEABLE</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>C (Pass / Reposition)</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>TRIGGERED</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Cheap CMMC-only self-serve tool: upload policies, auto gap-analysis + SPRS estimate + SSP/POA&amp;M; no consultant; competes head-on with FutureFeed/Vanta/Drata</t>
         </is>
       </c>
     </row>

</xml_diff>